<commit_message>
Atualiza textos e refina hub de ferramentas US Vale Verde
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -1,144 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferre\OneDrive\Documentos\PROJETOS PROGRAMAÇÃO\01. ENAEX\HUB DE FERRAMENTAS - US MVV\input\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F72B1C-FA6D-42CF-A1F4-420E418EC6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Repositorios" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t>Repositório</t>
-  </si>
-  <si>
-    <t>Título formal</t>
-  </si>
-  <si>
-    <t>GitHub</t>
-  </si>
-  <si>
-    <t>Pages</t>
-  </si>
-  <si>
-    <t>enaex-plano-de-voo</t>
-  </si>
-  <si>
-    <t>Conversor DXF para Poligonal no Google Earth com Exportação KMZ</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/enaex-plano-de-voo</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/enaex-plano-de-voo/</t>
-  </si>
-  <si>
-    <t>usmvv_planned_and_executed_data_consolidation</t>
-  </si>
-  <si>
-    <t>US Vale Verde PLAN/EXEC Data Console</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/usmvv_planned_and_executed_data_consolidation</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/usmvv_planned_and_executed_data_consolidation/</t>
-  </si>
-  <si>
-    <t>temposemovimentos</t>
-  </si>
-  <si>
-    <t>Sistema de Tempos e Movimentos</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/temposemovimentos</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/temposemovimentos/</t>
-  </si>
-  <si>
-    <t>blasthole-profile-creator</t>
-  </si>
-  <si>
-    <t>Blasthole Profile Creator</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/blasthole-profile-creator</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/blasthole-profile-creator/</t>
-  </si>
-  <si>
-    <t>pfr-enaex</t>
-  </si>
-  <si>
-    <t>PFR - Plano de Fogo Realizado</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/pfr-enaex</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/pfr-enaex/</t>
-  </si>
-  <si>
-    <t>aquickreportofseismographicdata</t>
-  </si>
-  <si>
-    <t>Report Sismografia Enaex</t>
-  </si>
-  <si>
-    <t>https://github.com/SILVAThiagoFerreira/aquickreportofseismographicdata</t>
-  </si>
-  <si>
-    <t>https://silvathiagoferreira.github.io/aquickreportofseismographicdata/</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <u/>
+      <name val="Arial"/>
+      <color rgb="FF0563C1"/>
       <sz val="10"/>
-      <color rgb="FF0563C1"/>
-      <name val="Arial"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -177,30 +83,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -488,127 +453,187 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58" customWidth="1"/>
-    <col min="3" max="4" width="68" customWidth="1"/>
+    <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Repositório</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Título formal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pages</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
+    <row r="2" ht="20.1" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>enaex-plano-de-voo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Conversor DXF para KMZ Operacional</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/enaex-plano-de-voo</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/enaex-plano-de-voo/</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
+    <row r="3" ht="20.1" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>usmvv_planned_and_executed_data_consolidation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Consolidação Plan./Exec. | US Vale Verde</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/usmvv_planned_and_executed_data_consolidation</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/usmvv_planned_and_executed_data_consolidation/</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
+    <row r="4" ht="20.1" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>temposemovimentos</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tempos e Movimentos | Carregamento de Explosivo</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/temposemovimentos</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/temposemovimentos/</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>19</v>
+    <row r="5" ht="20.1" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>blasthole-profile-creator</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Blasthole Profile Creator</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/blasthole-profile-creator</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/blasthole-profile-creator/</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>23</v>
+    <row r="6" ht="20.1" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>pfr-enaex</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PFR | Plano de Fogo Realizado</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/pfr-enaex</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/pfr-enaex/</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
+    <row r="7" ht="20.1" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>aquickreportofseismographicdata</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Report Sismografia Enaex</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/aquickreportofseismographicdata</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/aquickreportofseismographicdata/</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="C3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="D3" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="C4" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="D4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="C5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="D5" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="C6" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="D6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="C7" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="D7" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add public hub page to GitHub Pages project
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,50 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/correcao-de-cargas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>openblast-nbr9653</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>OpenBlast NBR 9653</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/openblast-nbr9653</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/openblast-nbr9653/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>conversor-pdf-seguro</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Conversor PDF Seguro</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/conversor-pdf-seguro</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/conversor-pdf-seguro/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza hubs e remove conversor PDF
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -683,28 +683,6 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/openblast-nbr9653/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>conversor-pdf-seguro</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Conversor PDF Seguro</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://github.com/SILVAThiagoFerreira/conversor-pdf-seguro</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://silvathiagoferreira.github.io/conversor-pdf-seguro/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add deviation analysis tool to both hubs
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,28 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/openblast-nbr9653/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>analise-de-desvios-de-inclinacao-e-azimute</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Análise de Desvios de Inclinação e Azimute</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/analise-de-desvios-de-inclinacao-e-azimute</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/analise-de-desvios-de-inclinacao-e-azimute/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rebrand hub manifests to openblast
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -491,7 +491,7 @@
     <row r="2" ht="20.1" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>enaex-plano-de-voo</t>
+          <t>openblast-plano-de-voo</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/SILVAThiagoFerreira/enaex-plano-de-voo</t>
+          <t>https://github.com/SILVAThiagoFerreira/openblast-plano-de-voo</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>https://silvathiagoferreira.github.io/enaex-plano-de-voo/</t>
+          <t>https://silvathiagoferreira.github.io/openblast-plano-de-voo/</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
     <row r="6" ht="20.1" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>pfr-enaex</t>
+          <t>pfr-openblast</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/SILVAThiagoFerreira/pfr-enaex</t>
+          <t>https://github.com/SILVAThiagoFerreira/pfr-openblast</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>https://silvathiagoferreira.github.io/pfr-enaex/</t>
+          <t>https://silvathiagoferreira.github.io/pfr-openblast/</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Report Sismografia Enaex</t>
+          <t>Report Sismografia OpenBlast</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix: align report sismografia repository links
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -601,7 +601,7 @@
     <row r="7" ht="20.1" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>aquickreportofseismographicdata</t>
+          <t>report-sismografia</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/SILVAThiagoFerreira/aquickreportofseismographicdata</t>
+          <t>https://github.com/SILVAThiagoFerreira/report-sismografia</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>https://silvathiagoferreira.github.io/aquickreportofseismographicdata/</t>
+          <t>https://silvathiagoferreira.github.io/report-sismografia/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza home do hub e publica manifesto filtrado
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -2,14 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -19,10 +15,8 @@
   <fonts count="4">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -39,7 +33,6 @@
       <name val="Arial"/>
       <color rgb="FF0563C1"/>
       <sz val="10"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,13 +49,7 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin">
         <color rgb="FFD9D9D9"/>
@@ -76,7 +63,6 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -95,9 +81,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -212,72 +197,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -333,7 +260,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -342,13 +269,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -382,17 +309,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -447,8 +363,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -461,7 +375,7 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="43.5703125" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="68" customWidth="1" min="3" max="4"/>
   </cols>
@@ -488,7 +402,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20.1" customHeight="1">
+    <row r="2" ht="20.10000038146973" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>openblast-plano-de-voo</t>
@@ -496,7 +410,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Conversor DXF para KMZ Operacional</t>
+          <t>Conversor: Boreholes/DXF para Limite DXF e KMZ (Plano de Voo)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -510,7 +424,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="20.1" customHeight="1">
+    <row r="3" ht="20.10000038146973" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>usmvv_planned_and_executed_data_consolidation</t>
@@ -532,7 +446,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20.1" customHeight="1">
+    <row r="4" ht="20.10000038146973" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>temposemovimentos</t>
@@ -554,7 +468,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="20.1" customHeight="1">
+    <row r="5" ht="20.10000038146973" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>blasthole-profile-creator</t>
@@ -576,7 +490,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20.1" customHeight="1">
+    <row r="6" ht="20.10000038146973" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>pfr-openblast</t>
@@ -598,7 +512,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20.1" customHeight="1">
+    <row r="7" ht="20.10000038146973" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>report-sismografia</t>
@@ -672,7 +586,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OpenBlast NBR 9653</t>
+          <t>ABNT NBR 9653*</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -723,6 +637,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: rename tool titles in hub
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Blasthole Profile Creator</t>
+          <t>Criador de Perfil de Furo de Desmonte</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Reporte de Sismografia</t>
+          <t>Report de Monitoramento Sismografico</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: add plano de fogo previsto to local tools hub
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -372,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" customWidth="1" min="1" max="1"/>
@@ -619,6 +619,28 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/analise-de-desvios-de-inclinacao-e-azimute/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20.10000038146973" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>plano-de-fogo-previsto</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Plano de Fogo Previsto</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/plano-de-fogo-previsto</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/plano-de-fogo-previsto/</t>
         </is>
       </c>
     </row>
@@ -636,6 +658,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>